<commit_message>
Atualizando o workspace e arquivos de configuração, incluindo a modificação do tipo e título da nota "Valores ODBC e Fechamento — Mapeamento de Colunas" para "Centro de Custo". Ajustando referências internas e removendo arquivos temporários obsoletos. Atualizando a nota "Critério de Rateio - Pilares" com informações detalhadas sobre a fórmula de rateio e percentuais por segmento, além de melhorias na formatação e inclusão de novas seções. Essas alterações visam aprimorar a clareza e a precisão das informações financeiras e operacionais.
</commit_message>
<xml_diff>
--- a/02-Referencias/ATUA/Abril/ATUA_despesas_fechamento_04-2026.xlsx
+++ b/02-Referencias/ATUA/Abril/ATUA_despesas_fechamento_04-2026.xlsx
@@ -946,17 +946,17 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>6.6.1</t>
+          <t>7.5.17</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>FRETE DE TERCEIROS</t>
+          <t>TAXAS</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>6.6.1 FRETE DE TERCEIROS</t>
+          <t>7.5.17 TAXAS</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -5500,17 +5500,17 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>6.6.1</t>
+          <t>7.5.17</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>FRETE DE TERCEIROS</t>
+          <t>TAXAS</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>6.6.1 FRETE DE TERCEIROS</t>
+          <t>7.5.17 TAXAS</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">

</xml_diff>